<commit_message>
fix: correct logic and add closing rate percentage
</commit_message>
<xml_diff>
--- a/DO/Rekap_Invoice_Konsultasi_Cleaned.xlsx
+++ b/DO/Rekap_Invoice_Konsultasi_Cleaned.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Documents\All Work Files\5. Main CLC Kemuning Kembar\DO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F2C3A5-B5A7-4508-A6BB-0361BBCE4C3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB9B0D6-79B6-4B33-925C-A1ECC3EAF546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$O$96</definedName>
+  </definedNames>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1012" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="362">
   <si>
     <t>Tanggal Payment</t>
   </si>
@@ -1103,6 +1106,9 @@
   </si>
   <si>
     <t>sesi sebelumnya di SOP dengan Psikolog Anggiastri Nama ortu: Nabsag Marlacuda Selawati</t>
+  </si>
+  <si>
+    <t>hitung unique value klien</t>
   </si>
 </sst>
 </file>
@@ -1127,7 +1133,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1142,6 +1148,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1173,7 +1185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1192,6 +1204,12 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1495,14 +1513,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O96"/>
+  <dimension ref="A1:O100"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="5" width="14.90625" customWidth="1"/>
+    <col min="5" max="5" width="23.90625" customWidth="1"/>
     <col min="6" max="6" width="23" customWidth="1"/>
     <col min="7" max="7" width="36" customWidth="1"/>
     <col min="8" max="8" width="19" customWidth="1"/>
@@ -5616,7 +5634,19 @@
         <v>52</v>
       </c>
     </row>
+    <row r="99" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E99" s="7" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="100" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E100" s="8">
+        <f>SUMPRODUCT(1/COUNTIF(D2:D20, D2:D20))</f>
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:O96" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add additional do
</commit_message>
<xml_diff>
--- a/DO/Rekap_Invoice_Konsultasi_Cleaned.xlsx
+++ b/DO/Rekap_Invoice_Konsultasi_Cleaned.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Documents\All Work Files\5. Main CLC Kemuning Kembar\DO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB9B0D6-79B6-4B33-925C-A1ECC3EAF546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC940E89-DA1E-43AB-A13F-99202E10A41D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="428">
   <si>
     <t>Tanggal Payment</t>
   </si>
@@ -1093,9 +1093,6 @@
     <t>sesi sebelumnya: 25 April 2026</t>
   </si>
   <si>
-    <t>17:20</t>
-  </si>
-  <si>
     <t>Alya Mukhbitah</t>
   </si>
   <si>
@@ -1105,10 +1102,211 @@
     <t>+628971999100(Marla)</t>
   </si>
   <si>
-    <t>sesi sebelumnya di SOP dengan Psikolog Anggiastri Nama ortu: Nabsag Marlacuda Selawati</t>
-  </si>
-  <si>
-    <t>hitung unique value klien</t>
+    <t>19:34</t>
+  </si>
+  <si>
+    <t>Anggita Susanti &amp; Andre</t>
+  </si>
+  <si>
+    <t>anggita.jevanjevin@gmail.com</t>
+  </si>
+  <si>
+    <t>+62817132559</t>
+  </si>
+  <si>
+    <t>Email Andre: andre0178@gmail.com</t>
+  </si>
+  <si>
+    <t>20:19</t>
+  </si>
+  <si>
+    <t>Mentari Sandiastri</t>
+  </si>
+  <si>
+    <t>sandiastri_mr@rocketmail.com</t>
+  </si>
+  <si>
+    <t>+6287782667164</t>
+  </si>
+  <si>
+    <t>18:52</t>
+  </si>
+  <si>
+    <t>+628971999100</t>
+  </si>
+  <si>
+    <t>1210</t>
+  </si>
+  <si>
+    <t>Tes Proyektif Anak</t>
+  </si>
+  <si>
+    <t>tes proyeksi (bhs Inggris) : 15.00-16.00 WIB : 480k sesi konsul ortu (bhs indo) : 16.00-17.00 WIB : 730k klien payment: 1,700k deposit: 490k</t>
+  </si>
+  <si>
+    <t>17:59</t>
+  </si>
+  <si>
+    <t>sesi sebelumnya : tes proyeksi : Sabtu, 2 Mei 2026 payment test proyeksi : 970.000 (sehingga ada sisa 490.000)</t>
+  </si>
+  <si>
+    <t>11:11</t>
+  </si>
+  <si>
+    <t>Claritza Prima Andana</t>
+  </si>
+  <si>
+    <t>sekarhastari@gmail.com</t>
+  </si>
+  <si>
+    <t>+6281218889049</t>
+  </si>
+  <si>
+    <t>Nama Orang Tua : Priyandana dan Sekar Hastari sesi 2 : TBC</t>
+  </si>
+  <si>
+    <t>16:46</t>
+  </si>
+  <si>
+    <t>Liza Erica Panjaitan</t>
+  </si>
+  <si>
+    <t>lizaerica@gmail.com</t>
+  </si>
+  <si>
+    <t>+6282233648955</t>
+  </si>
+  <si>
+    <t>Hipnoterapi</t>
+  </si>
+  <si>
+    <t>17:12</t>
+  </si>
+  <si>
+    <t>16:47</t>
+  </si>
+  <si>
+    <t>Nurmah Rabbyyatna</t>
+  </si>
+  <si>
+    <t>nrabbyyatnasari@gmail.com</t>
+  </si>
+  <si>
+    <t>+6281286426750</t>
+  </si>
+  <si>
+    <t>11:54</t>
+  </si>
+  <si>
+    <t>+60173553802</t>
+  </si>
+  <si>
+    <t>sesi sebelumnya: 4 Mei 2026</t>
+  </si>
+  <si>
+    <t>19:03</t>
+  </si>
+  <si>
+    <t>1380</t>
+  </si>
+  <si>
+    <t>21:06</t>
+  </si>
+  <si>
+    <t>sesi sebelumnya: 27 April 2026</t>
+  </si>
+  <si>
+    <t>09:18</t>
+  </si>
+  <si>
+    <t>sesi sebelumnya: 9 April 2026</t>
+  </si>
+  <si>
+    <t>07:58</t>
+  </si>
+  <si>
+    <t>Nathania Hasna Griselda</t>
+  </si>
+  <si>
+    <t>nikenpurwadi@gmail.com</t>
+  </si>
+  <si>
+    <t>+6285893182278</t>
+  </si>
+  <si>
+    <t>10:46</t>
+  </si>
+  <si>
+    <t>Salomo Maurice Angelo</t>
+  </si>
+  <si>
+    <t>klien merupakan anak dari klien Danielli Amanda Luvita (11 April) sesi 2: tbc</t>
+  </si>
+  <si>
+    <t>13:28</t>
+  </si>
+  <si>
+    <t>sesi sebelumnya: 7 Mei 2026</t>
+  </si>
+  <si>
+    <t>14:12</t>
+  </si>
+  <si>
+    <t>Emboyo Retno</t>
+  </si>
+  <si>
+    <t>Klien merupakan Ibu dari klien Anggita Nuraini</t>
+  </si>
+  <si>
+    <t>14:17</t>
+  </si>
+  <si>
+    <t>Gunawan Aji Putranto</t>
+  </si>
+  <si>
+    <t>Klien merupakan Ayah dari klien Anggita Nuraini</t>
+  </si>
+  <si>
+    <t>09:33</t>
+  </si>
+  <si>
+    <t>Wisnu Brata Dasuki</t>
+  </si>
+  <si>
+    <t>wisnubrata.dasuki@gmail.com</t>
+  </si>
+  <si>
+    <t>+6287784452268</t>
+  </si>
+  <si>
+    <t>570</t>
+  </si>
+  <si>
+    <t>Tes Intelegensi Dewasa</t>
+  </si>
+  <si>
+    <t>15:15</t>
+  </si>
+  <si>
+    <t>Vino Devano Darma Lian</t>
+  </si>
+  <si>
+    <t>supriatiningsihupi@yahoo.com</t>
+  </si>
+  <si>
+    <t>+628118336508</t>
+  </si>
+  <si>
+    <t>Tes Persiapan Sekolah Individual</t>
+  </si>
+  <si>
+    <t>Nama Ayah: Dedy Lian Nama Ibu: Supriatiningsih</t>
+  </si>
+  <si>
+    <t>12:07</t>
+  </si>
+  <si>
+    <t>sesi sebelumnya: 12 Februari 2026</t>
   </si>
 </sst>
 </file>
@@ -1118,7 +1316,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1132,8 +1330,14 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1151,12 +1355,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1168,16 +1366,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1205,11 +1403,11 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1513,7 +1711,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O100"/>
+  <dimension ref="A1:O116"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -1529,7 +1727,8 @@
     <col min="11" max="11" width="17" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
     <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="15" width="40" customWidth="1"/>
+    <col min="14" max="14" width="40" customWidth="1"/>
+    <col min="15" max="15" width="43.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -5350,7 +5549,9 @@
       <c r="D90" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="E90" s="5"/>
+      <c r="E90" s="7" t="s">
+        <v>349</v>
+      </c>
       <c r="F90" s="6"/>
       <c r="G90" s="3" t="s">
         <v>282</v>
@@ -5595,27 +5796,29 @@
     </row>
     <row r="96" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C96" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="E96" s="5"/>
-      <c r="F96" s="3"/>
+        <v>360</v>
+      </c>
+      <c r="E96" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="F96" s="5"/>
       <c r="G96" s="3" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="I96" s="3" t="s">
-        <v>18</v>
+        <v>64</v>
       </c>
       <c r="J96" s="3">
         <v>1</v>
@@ -5624,29 +5827,877 @@
         <v>19</v>
       </c>
       <c r="L96" s="3" t="s">
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="M96" s="3"/>
       <c r="N96" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="O96" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A97" s="2">
+        <v>46142</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="E97" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F97" s="3"/>
+      <c r="G97" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="H97" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="I97" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="J97" s="3">
+        <v>1</v>
+      </c>
+      <c r="K97" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L97" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M97" s="3"/>
+      <c r="N97" s="3"/>
+      <c r="O97" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="98" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A98" s="2">
+        <v>46142</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="E98" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="H98" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="I98" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="J98" s="3">
+        <v>1</v>
+      </c>
+      <c r="K98" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L98" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="M98" s="3"/>
+      <c r="N98" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="O98" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A99" s="2">
+        <v>46145</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F99" s="3"/>
+      <c r="G99" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="H99" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="I99" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="J99" s="3">
+        <v>1</v>
+      </c>
+      <c r="K99" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L99" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M99" s="3"/>
+      <c r="N99" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="O99" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A100" s="2">
+        <v>46147</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="E100" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="F100" s="6">
+        <v>46145</v>
+      </c>
+      <c r="G100" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="H100" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="I100" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J100" s="3">
+        <v>1</v>
+      </c>
+      <c r="K100" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L100" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="M100" s="3"/>
+      <c r="N100" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="O100" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A101" s="2">
+        <v>46148</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="E101" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="F101" s="6">
+        <v>46141</v>
+      </c>
+      <c r="G101" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="H101" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="I101" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="J101" s="3">
+        <v>1</v>
+      </c>
+      <c r="K101" s="3"/>
+      <c r="L101" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="M101" s="3"/>
+      <c r="N101" s="3"/>
+      <c r="O101" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A102" s="2">
+        <v>46149</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="E102" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F102" s="3"/>
+      <c r="G102" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="H102" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I102" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J102" s="3">
+        <v>1</v>
+      </c>
+      <c r="K102" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L102" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M102" s="3"/>
+      <c r="N102" s="3"/>
+      <c r="O102" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A103" s="2">
+        <v>46149</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E103" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="F103" s="6">
+        <v>46149</v>
+      </c>
+      <c r="G103" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="H103" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="I103" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J103" s="3">
+        <v>1</v>
+      </c>
+      <c r="K103" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L103" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M103" s="3"/>
+      <c r="N103" s="3"/>
+      <c r="O103" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A104" s="2">
+        <v>46150</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F104" s="3"/>
+      <c r="G104" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="H104" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="I104" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J104" s="3">
+        <v>1</v>
+      </c>
+      <c r="K104" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L104" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="M104" s="3"/>
+      <c r="N104" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="O104" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="105" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A105" s="2">
+        <v>46151</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="E105" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F105" s="3"/>
+      <c r="G105" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="H105" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="I105" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="J105" s="3">
+        <v>1</v>
+      </c>
+      <c r="K105" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L105" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="M105" s="3"/>
+      <c r="N105" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="O105" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="106" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A106" s="2">
+        <v>46153</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F106" s="3"/>
+      <c r="G106" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="H106" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="I106" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J106" s="3">
+        <v>1</v>
+      </c>
+      <c r="K106" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L106" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M106" s="3"/>
+      <c r="N106" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="O106" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="107" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A107" s="2">
+        <v>46154</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F107" s="3"/>
+      <c r="G107" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="H107" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="I107" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J107" s="3">
+        <v>1</v>
+      </c>
+      <c r="K107" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L107" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M107" s="3"/>
+      <c r="N107" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="O107" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="108" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A108" s="2">
+        <v>46154</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="E108" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="F108" s="6">
+        <v>46154</v>
+      </c>
+      <c r="G108" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="H108" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="I108" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J108" s="3">
+        <v>1</v>
+      </c>
+      <c r="K108" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L108" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M108" s="3"/>
+      <c r="N108" s="3"/>
+      <c r="O108" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="109" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A109" s="2">
+        <v>46155</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="E109" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="F109" s="3"/>
+      <c r="G109" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H109" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="I109" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J109" s="3">
+        <v>1</v>
+      </c>
+      <c r="K109" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L109" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="M109" s="3"/>
+      <c r="N109" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="O109" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="110" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A110" s="2">
+        <v>46155</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="E110" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F110" s="3"/>
+      <c r="G110" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="H110" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="I110" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="J110" s="3">
+        <v>1</v>
+      </c>
+      <c r="K110" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L110" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M110" s="3"/>
+      <c r="N110" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="O110" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="111" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A111" s="2">
+        <v>46156</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D111" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="O96" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="99" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E99" s="7" t="s">
+      <c r="E111" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F111" s="3"/>
+      <c r="G111" s="3" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="100" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E100" s="8">
-        <f>SUMPRODUCT(1/COUNTIF(D2:D20, D2:D20))</f>
-        <v>13</v>
+      <c r="H111" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="I111" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="J111" s="3">
+        <v>1</v>
+      </c>
+      <c r="K111" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L111" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="M111" s="3"/>
+      <c r="N111" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="O111" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="112" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A112" s="2">
+        <v>46161</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="E112" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="F112" s="3"/>
+      <c r="G112" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="H112" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="I112" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J112" s="3">
+        <v>1</v>
+      </c>
+      <c r="K112" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L112" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M112" s="3"/>
+      <c r="N112" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="O112" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="113" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A113" s="2">
+        <v>46161</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="F113" s="3"/>
+      <c r="G113" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="H113" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="I113" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J113" s="3">
+        <v>1</v>
+      </c>
+      <c r="K113" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L113" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M113" s="3"/>
+      <c r="N113" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="O113" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="114" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A114" s="2">
+        <v>46161</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D114" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="E114" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="F114" s="6">
+        <v>46160</v>
+      </c>
+      <c r="G114" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="H114" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="I114" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="J114" s="3">
+        <v>1</v>
+      </c>
+      <c r="K114" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L114" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="M114" s="3"/>
+      <c r="N114" s="3"/>
+      <c r="O114" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="115" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A115" s="2">
+        <v>46161</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E115" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="F115" s="6">
+        <v>46161</v>
+      </c>
+      <c r="G115" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="H115" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="I115" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J115" s="3">
+        <v>1</v>
+      </c>
+      <c r="K115" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L115" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="M115" s="3"/>
+      <c r="N115" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="O115" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="116" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A116" s="2">
+        <v>46150</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E116" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F116" s="3"/>
+      <c r="G116" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="H116" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="I116" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J116" s="3">
+        <v>1</v>
+      </c>
+      <c r="K116" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L116" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M116" s="3"/>
+      <c r="N116" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="O116" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O96" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>